<commit_message>
Update loginAdmin to read Sheet2, add loginAdmin project config
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NIC\Desktop\Test_2nd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{720E99C8-019E-45C4-8D0C-F804135F65BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68A71FF5-BEB2-4DDA-B8D6-8B6DADE1AEA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{0DDFC77C-2A2E-493A-915B-2CC1D18DEEE1}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
   <si>
     <t>username</t>
   </si>
@@ -38,6 +38,15 @@
   </si>
   <si>
     <t>123456Aa@</t>
+  </si>
+  <si>
+    <t>long4</t>
+  </si>
+  <si>
+    <t>long3</t>
+  </si>
+  <si>
+    <t>tuan1</t>
   </si>
 </sst>
 </file>
@@ -423,9 +432,17 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B3" s="1"/>
+      <c r="A3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
@@ -434,6 +451,7 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{9D6DCD52-6267-49A7-8213-FFAEE9516BF3}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{65A1E35C-29F5-4245-8B4C-1A3921D815ED}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -458,7 +476,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
Update test results, storage states, and remove createaccount test
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NIC\Desktop\Test_2nd\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68A71FF5-BEB2-4DDA-B8D6-8B6DADE1AEA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{799E087A-5400-42C7-A7AD-840D8F22434C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{0DDFC77C-2A2E-493A-915B-2CC1D18DEEE1}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{0DDFC77C-2A2E-493A-915B-2CC1D18DEEE1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -26,27 +26,27 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="7">
   <si>
     <t>username</t>
   </si>
   <si>
-    <t>long5</t>
-  </si>
-  <si>
     <t>password</t>
   </si>
   <si>
     <t>123456Aa@</t>
   </si>
   <si>
-    <t>long4</t>
-  </si>
-  <si>
-    <t>long3</t>
-  </si>
-  <si>
-    <t>tuan1</t>
+    <t>truong1</t>
+  </si>
+  <si>
+    <t>truong2</t>
+  </si>
+  <si>
+    <t>truong</t>
+  </si>
+  <si>
+    <t>truong3</t>
   </si>
 </sst>
 </file>
@@ -420,15 +420,15 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -436,22 +436,25 @@
         <v>4</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{9D6DCD52-6267-49A7-8213-FFAEE9516BF3}"/>
-    <hyperlink ref="B3" r:id="rId2" xr:uid="{65A1E35C-29F5-4245-8B4C-1A3921D815ED}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{65A1E35C-29F5-4245-8B4C-1A3921D815ED}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{6310BE95-78EB-4B79-8BE4-DD4BE97A3550}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -471,15 +474,15 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>